<commit_message>
Final commit for safety experimentation
</commit_message>
<xml_diff>
--- a/Research_Daily_Plan.xlsx
+++ b/Research_Daily_Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rahul\Nyaymalaw 3.0\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D592E86-519D-4C8B-914E-299FD7A2B457}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45B471D0-55E4-47A3-93C1-DE6ACA59CF5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1370,7 +1370,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1383,6 +1383,9 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1864,7 +1867,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" ht="112.2" x14ac:dyDescent="0.3">
       <c r="A5" s="5">
         <v>1</v>
       </c>
@@ -1874,20 +1877,20 @@
       <c r="C5" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="38">
+      <c r="D5" s="39">
         <v>46072</v>
       </c>
       <c r="E5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="F5" s="39" t="s">
+      <c r="F5" s="40" t="s">
         <v>13</v>
       </c>
       <c r="G5" s="5">
         <v>2</v>
       </c>
       <c r="H5" s="5"/>
-      <c r="I5" s="40" t="s">
+      <c r="I5" s="7" t="s">
         <v>14</v>
       </c>
       <c r="J5" s="5" t="s">
@@ -1904,14 +1907,14 @@
       <c r="C6" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="38">
+      <c r="D6" s="39">
         <f>D5+1</f>
         <v>46073</v>
       </c>
       <c r="E6" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="F6" s="39" t="s">
+      <c r="F6" s="40" t="s">
         <v>17</v>
       </c>
       <c r="G6" s="5">
@@ -1920,7 +1923,7 @@
       <c r="H6" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="I6" s="40" t="s">
+      <c r="I6" s="41" t="s">
         <v>18</v>
       </c>
       <c r="J6" s="5" t="s">
@@ -1937,21 +1940,21 @@
       <c r="C7" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="D7" s="38">
+      <c r="D7" s="39">
         <f t="shared" ref="D7:D69" si="0">D6+1</f>
         <v>46074</v>
       </c>
       <c r="E7" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="F7" s="39" t="s">
+      <c r="F7" s="40" t="s">
         <v>20</v>
       </c>
       <c r="G7" s="5">
         <v>2</v>
       </c>
       <c r="H7" s="5"/>
-      <c r="I7" s="40" t="s">
+      <c r="I7" s="41" t="s">
         <v>21</v>
       </c>
       <c r="J7" s="5" t="s">
@@ -1968,21 +1971,21 @@
       <c r="C8" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="D8" s="38">
+      <c r="D8" s="39">
         <f t="shared" si="0"/>
         <v>46075</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="F8" s="39" t="s">
+      <c r="F8" s="40" t="s">
         <v>23</v>
       </c>
       <c r="G8" s="5">
         <v>2</v>
       </c>
       <c r="H8" s="5"/>
-      <c r="I8" s="40" t="s">
+      <c r="I8" s="41" t="s">
         <v>24</v>
       </c>
       <c r="J8" s="5" t="s">
@@ -1990,1905 +1993,1905 @@
       </c>
     </row>
     <row r="9" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A9" s="7">
+      <c r="A9" s="8">
         <v>5</v>
       </c>
-      <c r="B9" s="7">
+      <c r="B9" s="8">
         <v>1</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C9" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="D9" s="38">
+      <c r="D9" s="39">
         <f t="shared" si="0"/>
         <v>46076</v>
       </c>
-      <c r="E9" s="8" t="s">
+      <c r="E9" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="F9" s="41" t="s">
+      <c r="F9" s="42" t="s">
         <v>27</v>
       </c>
-      <c r="G9" s="7">
-        <v>2</v>
-      </c>
-      <c r="H9" s="7"/>
-      <c r="I9" s="42" t="s">
+      <c r="G9" s="8">
+        <v>2</v>
+      </c>
+      <c r="H9" s="8"/>
+      <c r="I9" s="43" t="s">
         <v>28</v>
       </c>
-      <c r="J9" s="7" t="s">
+      <c r="J9" s="8" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A10" s="9">
+      <c r="A10" s="10">
         <v>6</v>
       </c>
-      <c r="B10" s="9">
+      <c r="B10" s="10">
         <v>1</v>
       </c>
-      <c r="C10" s="9" t="s">
+      <c r="C10" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="D10" s="38">
+      <c r="D10" s="39">
         <f t="shared" si="0"/>
         <v>46077</v>
       </c>
-      <c r="E10" s="10" t="s">
+      <c r="E10" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="F10" s="43" t="s">
+      <c r="F10" s="44" t="s">
         <v>30</v>
       </c>
-      <c r="G10" s="9">
+      <c r="G10" s="10">
         <v>5</v>
       </c>
-      <c r="H10" s="9"/>
-      <c r="I10" s="44" t="s">
+      <c r="H10" s="10"/>
+      <c r="I10" s="45" t="s">
         <v>31</v>
       </c>
-      <c r="J10" s="9" t="s">
+      <c r="J10" s="10" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A11" s="9">
+      <c r="A11" s="10">
         <v>7</v>
       </c>
-      <c r="B11" s="9">
+      <c r="B11" s="10">
         <v>1</v>
       </c>
-      <c r="C11" s="9" t="s">
+      <c r="C11" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="D11" s="38">
+      <c r="D11" s="39">
         <f t="shared" si="0"/>
         <v>46078</v>
       </c>
-      <c r="E11" s="10" t="s">
+      <c r="E11" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="F11" s="43" t="s">
+      <c r="F11" s="44" t="s">
         <v>33</v>
       </c>
-      <c r="G11" s="9">
+      <c r="G11" s="10">
         <v>5</v>
       </c>
-      <c r="H11" s="9"/>
-      <c r="I11" s="44" t="s">
+      <c r="H11" s="10"/>
+      <c r="I11" s="45" t="s">
         <v>34</v>
       </c>
-      <c r="J11" s="9" t="s">
+      <c r="J11" s="10" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A12" s="7">
+      <c r="A12" s="8">
         <v>8</v>
       </c>
-      <c r="B12" s="7">
-        <v>2</v>
-      </c>
-      <c r="C12" s="7" t="s">
+      <c r="B12" s="8">
+        <v>2</v>
+      </c>
+      <c r="C12" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="D12" s="38">
+      <c r="D12" s="39">
         <f t="shared" si="0"/>
         <v>46079</v>
       </c>
-      <c r="E12" s="8" t="s">
+      <c r="E12" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="F12" s="41" t="s">
+      <c r="F12" s="42" t="s">
         <v>35</v>
       </c>
-      <c r="G12" s="7">
-        <v>2</v>
-      </c>
-      <c r="H12" s="7"/>
-      <c r="I12" s="42" t="s">
+      <c r="G12" s="8">
+        <v>2</v>
+      </c>
+      <c r="H12" s="8"/>
+      <c r="I12" s="43" t="s">
         <v>36</v>
       </c>
-      <c r="J12" s="7" t="s">
+      <c r="J12" s="8" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A13" s="7">
+      <c r="A13" s="8">
         <v>9</v>
       </c>
-      <c r="B13" s="7">
-        <v>2</v>
-      </c>
-      <c r="C13" s="7" t="s">
+      <c r="B13" s="8">
+        <v>2</v>
+      </c>
+      <c r="C13" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="D13" s="38">
+      <c r="D13" s="39">
         <f t="shared" si="0"/>
         <v>46080</v>
       </c>
-      <c r="E13" s="8" t="s">
+      <c r="E13" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="F13" s="41" t="s">
+      <c r="F13" s="42" t="s">
         <v>37</v>
       </c>
-      <c r="G13" s="7">
-        <v>2</v>
-      </c>
-      <c r="H13" s="7"/>
-      <c r="I13" s="42" t="s">
+      <c r="G13" s="8">
+        <v>2</v>
+      </c>
+      <c r="H13" s="8"/>
+      <c r="I13" s="43" t="s">
         <v>38</v>
       </c>
-      <c r="J13" s="7" t="s">
+      <c r="J13" s="8" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A14" s="7">
+      <c r="A14" s="8">
         <v>10</v>
       </c>
-      <c r="B14" s="7">
-        <v>2</v>
-      </c>
-      <c r="C14" s="7" t="s">
+      <c r="B14" s="8">
+        <v>2</v>
+      </c>
+      <c r="C14" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="D14" s="38">
+      <c r="D14" s="39">
         <f t="shared" si="0"/>
         <v>46081</v>
       </c>
-      <c r="E14" s="8" t="s">
+      <c r="E14" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="F14" s="41" t="s">
+      <c r="F14" s="42" t="s">
         <v>39</v>
       </c>
-      <c r="G14" s="7">
-        <v>2</v>
-      </c>
-      <c r="H14" s="7"/>
-      <c r="I14" s="42" t="s">
+      <c r="G14" s="8">
+        <v>2</v>
+      </c>
+      <c r="H14" s="8"/>
+      <c r="I14" s="43" t="s">
         <v>40</v>
       </c>
-      <c r="J14" s="7" t="s">
+      <c r="J14" s="8" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A15" s="7">
+      <c r="A15" s="8">
         <v>11</v>
       </c>
-      <c r="B15" s="7">
-        <v>2</v>
-      </c>
-      <c r="C15" s="7" t="s">
+      <c r="B15" s="8">
+        <v>2</v>
+      </c>
+      <c r="C15" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="D15" s="38">
+      <c r="D15" s="39">
         <f t="shared" si="0"/>
         <v>46082</v>
       </c>
-      <c r="E15" s="8" t="s">
+      <c r="E15" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="F15" s="41" t="s">
+      <c r="F15" s="42" t="s">
         <v>41</v>
       </c>
-      <c r="G15" s="7">
-        <v>2</v>
-      </c>
-      <c r="H15" s="7"/>
-      <c r="I15" s="42" t="s">
+      <c r="G15" s="8">
+        <v>2</v>
+      </c>
+      <c r="H15" s="8"/>
+      <c r="I15" s="43" t="s">
         <v>42</v>
       </c>
-      <c r="J15" s="7" t="s">
+      <c r="J15" s="8" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A16" s="7">
+      <c r="A16" s="8">
         <v>12</v>
       </c>
-      <c r="B16" s="7">
-        <v>2</v>
-      </c>
-      <c r="C16" s="7" t="s">
+      <c r="B16" s="8">
+        <v>2</v>
+      </c>
+      <c r="C16" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="D16" s="38">
+      <c r="D16" s="39">
         <f t="shared" si="0"/>
         <v>46083</v>
       </c>
-      <c r="E16" s="8" t="s">
+      <c r="E16" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="F16" s="41" t="s">
+      <c r="F16" s="42" t="s">
         <v>43</v>
       </c>
-      <c r="G16" s="7">
-        <v>2</v>
-      </c>
-      <c r="H16" s="7"/>
-      <c r="I16" s="42" t="s">
+      <c r="G16" s="8">
+        <v>2</v>
+      </c>
+      <c r="H16" s="8"/>
+      <c r="I16" s="43" t="s">
         <v>44</v>
       </c>
-      <c r="J16" s="7" t="s">
+      <c r="J16" s="8" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A17" s="9">
+      <c r="A17" s="10">
         <v>13</v>
       </c>
-      <c r="B17" s="9">
-        <v>2</v>
-      </c>
-      <c r="C17" s="9" t="s">
+      <c r="B17" s="10">
+        <v>2</v>
+      </c>
+      <c r="C17" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="D17" s="38">
+      <c r="D17" s="39">
         <f t="shared" si="0"/>
         <v>46084</v>
       </c>
-      <c r="E17" s="10" t="s">
+      <c r="E17" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="F17" s="43" t="s">
+      <c r="F17" s="44" t="s">
         <v>45</v>
       </c>
-      <c r="G17" s="9">
+      <c r="G17" s="10">
         <v>5</v>
       </c>
-      <c r="H17" s="9"/>
-      <c r="I17" s="44" t="s">
+      <c r="H17" s="10"/>
+      <c r="I17" s="45" t="s">
         <v>46</v>
       </c>
-      <c r="J17" s="9" t="s">
+      <c r="J17" s="10" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="18" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A18" s="9">
+      <c r="A18" s="10">
         <v>14</v>
       </c>
-      <c r="B18" s="9">
-        <v>2</v>
-      </c>
-      <c r="C18" s="9" t="s">
+      <c r="B18" s="10">
+        <v>2</v>
+      </c>
+      <c r="C18" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="D18" s="38">
+      <c r="D18" s="39">
         <f t="shared" si="0"/>
         <v>46085</v>
       </c>
-      <c r="E18" s="10" t="s">
+      <c r="E18" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="F18" s="43" t="s">
+      <c r="F18" s="44" t="s">
         <v>48</v>
       </c>
-      <c r="G18" s="9">
+      <c r="G18" s="10">
         <v>5</v>
       </c>
-      <c r="H18" s="9" t="s">
+      <c r="H18" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="I18" s="44" t="s">
+      <c r="I18" s="45" t="s">
         <v>49</v>
       </c>
-      <c r="J18" s="9" t="s">
+      <c r="J18" s="10" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="19" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A19" s="7">
-        <v>15</v>
-      </c>
-      <c r="B19" s="7">
+      <c r="A19" s="8">
+        <v>15</v>
+      </c>
+      <c r="B19" s="8">
         <v>3</v>
       </c>
-      <c r="C19" s="7" t="s">
+      <c r="C19" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="D19" s="38">
+      <c r="D19" s="39">
         <f t="shared" si="0"/>
         <v>46086</v>
       </c>
-      <c r="E19" s="8" t="s">
+      <c r="E19" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="F19" s="41" t="s">
+      <c r="F19" s="42" t="s">
         <v>50</v>
       </c>
-      <c r="G19" s="7">
-        <v>2</v>
-      </c>
-      <c r="H19" s="7"/>
-      <c r="I19" s="42" t="s">
+      <c r="G19" s="8">
+        <v>2</v>
+      </c>
+      <c r="H19" s="8"/>
+      <c r="I19" s="43" t="s">
         <v>51</v>
       </c>
-      <c r="J19" s="7" t="s">
+      <c r="J19" s="8" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="20" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A20" s="7">
+      <c r="A20" s="8">
         <v>16</v>
       </c>
-      <c r="B20" s="7">
+      <c r="B20" s="8">
         <v>3</v>
       </c>
-      <c r="C20" s="7" t="s">
+      <c r="C20" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="D20" s="38">
+      <c r="D20" s="39">
         <f t="shared" si="0"/>
         <v>46087</v>
       </c>
-      <c r="E20" s="8" t="s">
+      <c r="E20" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="F20" s="41" t="s">
+      <c r="F20" s="42" t="s">
         <v>52</v>
       </c>
-      <c r="G20" s="7">
-        <v>2</v>
-      </c>
-      <c r="H20" s="7"/>
-      <c r="I20" s="42" t="s">
+      <c r="G20" s="8">
+        <v>2</v>
+      </c>
+      <c r="H20" s="8"/>
+      <c r="I20" s="43" t="s">
         <v>53</v>
       </c>
-      <c r="J20" s="7" t="s">
+      <c r="J20" s="8" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="21" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A21" s="7">
+      <c r="A21" s="8">
         <v>17</v>
       </c>
-      <c r="B21" s="7">
+      <c r="B21" s="8">
         <v>3</v>
       </c>
-      <c r="C21" s="7" t="s">
+      <c r="C21" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="D21" s="38">
+      <c r="D21" s="39">
         <f t="shared" si="0"/>
         <v>46088</v>
       </c>
-      <c r="E21" s="8" t="s">
+      <c r="E21" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="F21" s="41" t="s">
+      <c r="F21" s="42" t="s">
         <v>54</v>
       </c>
-      <c r="G21" s="7">
-        <v>2</v>
-      </c>
-      <c r="H21" s="7"/>
-      <c r="I21" s="42" t="s">
+      <c r="G21" s="8">
+        <v>2</v>
+      </c>
+      <c r="H21" s="8"/>
+      <c r="I21" s="43" t="s">
         <v>55</v>
       </c>
-      <c r="J21" s="7" t="s">
+      <c r="J21" s="8" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="22" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A22" s="11">
+      <c r="A22" s="12">
         <v>18</v>
       </c>
-      <c r="B22" s="11">
+      <c r="B22" s="12">
         <v>3</v>
       </c>
-      <c r="C22" s="11" t="s">
+      <c r="C22" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="D22" s="38">
+      <c r="D22" s="39">
         <f t="shared" si="0"/>
         <v>46089</v>
       </c>
-      <c r="E22" s="12" t="s">
+      <c r="E22" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="F22" s="45" t="s">
+      <c r="F22" s="46" t="s">
         <v>57</v>
       </c>
-      <c r="G22" s="11">
-        <v>2</v>
-      </c>
-      <c r="H22" s="11"/>
-      <c r="I22" s="46" t="s">
+      <c r="G22" s="12">
+        <v>2</v>
+      </c>
+      <c r="H22" s="12"/>
+      <c r="I22" s="47" t="s">
         <v>58</v>
       </c>
-      <c r="J22" s="11" t="s">
+      <c r="J22" s="12" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="23" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A23" s="13">
+      <c r="A23" s="14">
         <v>19</v>
       </c>
-      <c r="B23" s="13">
+      <c r="B23" s="14">
         <v>3</v>
       </c>
-      <c r="C23" s="13" t="s">
+      <c r="C23" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="D23" s="38">
+      <c r="D23" s="39">
         <f t="shared" si="0"/>
         <v>46090</v>
       </c>
-      <c r="E23" s="14" t="s">
+      <c r="E23" s="15" t="s">
         <v>47</v>
       </c>
-      <c r="F23" s="47" t="s">
+      <c r="F23" s="48" t="s">
         <v>59</v>
       </c>
-      <c r="G23" s="13">
-        <v>2</v>
-      </c>
-      <c r="H23" s="13" t="s">
+      <c r="G23" s="14">
+        <v>2</v>
+      </c>
+      <c r="H23" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="I23" s="48" t="s">
+      <c r="I23" s="49" t="s">
         <v>60</v>
       </c>
-      <c r="J23" s="13" t="s">
+      <c r="J23" s="14" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="24" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A24" s="9">
+      <c r="A24" s="10">
         <v>20</v>
       </c>
-      <c r="B24" s="9">
+      <c r="B24" s="10">
         <v>3</v>
       </c>
-      <c r="C24" s="9" t="s">
+      <c r="C24" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="D24" s="38">
+      <c r="D24" s="39">
         <f t="shared" si="0"/>
         <v>46091</v>
       </c>
-      <c r="E24" s="10" t="s">
+      <c r="E24" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="F24" s="43" t="s">
+      <c r="F24" s="44" t="s">
         <v>61</v>
       </c>
-      <c r="G24" s="9">
+      <c r="G24" s="10">
         <v>5</v>
       </c>
-      <c r="H24" s="9"/>
-      <c r="I24" s="44" t="s">
+      <c r="H24" s="10"/>
+      <c r="I24" s="45" t="s">
         <v>62</v>
       </c>
-      <c r="J24" s="9" t="s">
+      <c r="J24" s="10" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="25" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A25" s="9">
+      <c r="A25" s="10">
         <v>21</v>
       </c>
-      <c r="B25" s="9">
+      <c r="B25" s="10">
         <v>3</v>
       </c>
-      <c r="C25" s="9" t="s">
+      <c r="C25" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="D25" s="38">
+      <c r="D25" s="39">
         <f t="shared" si="0"/>
         <v>46092</v>
       </c>
-      <c r="E25" s="10" t="s">
+      <c r="E25" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="F25" s="43" t="s">
+      <c r="F25" s="44" t="s">
         <v>63</v>
       </c>
-      <c r="G25" s="9">
+      <c r="G25" s="10">
         <v>5</v>
       </c>
-      <c r="H25" s="9"/>
-      <c r="I25" s="44" t="s">
+      <c r="H25" s="10"/>
+      <c r="I25" s="45" t="s">
         <v>64</v>
       </c>
-      <c r="J25" s="9" t="s">
+      <c r="J25" s="10" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="26" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A26" s="13">
+      <c r="A26" s="14">
         <v>22</v>
       </c>
-      <c r="B26" s="13">
+      <c r="B26" s="14">
         <v>4</v>
       </c>
-      <c r="C26" s="13" t="s">
+      <c r="C26" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="D26" s="38">
+      <c r="D26" s="39">
         <f t="shared" si="0"/>
         <v>46093</v>
       </c>
-      <c r="E26" s="14" t="s">
+      <c r="E26" s="15" t="s">
         <v>47</v>
       </c>
-      <c r="F26" s="47" t="s">
+      <c r="F26" s="48" t="s">
         <v>65</v>
       </c>
-      <c r="G26" s="13">
-        <v>2</v>
-      </c>
-      <c r="H26" s="13"/>
-      <c r="I26" s="48" t="s">
+      <c r="G26" s="14">
+        <v>2</v>
+      </c>
+      <c r="H26" s="14"/>
+      <c r="I26" s="49" t="s">
         <v>66</v>
       </c>
-      <c r="J26" s="13" t="s">
+      <c r="J26" s="14" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="27" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A27" s="13">
+      <c r="A27" s="14">
         <v>23</v>
       </c>
-      <c r="B27" s="13">
+      <c r="B27" s="14">
         <v>4</v>
       </c>
-      <c r="C27" s="13" t="s">
+      <c r="C27" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="D27" s="38">
+      <c r="D27" s="39">
         <f t="shared" si="0"/>
         <v>46094</v>
       </c>
-      <c r="E27" s="14" t="s">
+      <c r="E27" s="15" t="s">
         <v>47</v>
       </c>
-      <c r="F27" s="47" t="s">
+      <c r="F27" s="48" t="s">
         <v>67</v>
       </c>
-      <c r="G27" s="13">
-        <v>2</v>
-      </c>
-      <c r="H27" s="13"/>
-      <c r="I27" s="48" t="s">
+      <c r="G27" s="14">
+        <v>2</v>
+      </c>
+      <c r="H27" s="14"/>
+      <c r="I27" s="49" t="s">
         <v>68</v>
       </c>
-      <c r="J27" s="13" t="s">
+      <c r="J27" s="14" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="28" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A28" s="15">
+      <c r="A28" s="16">
         <v>24</v>
       </c>
-      <c r="B28" s="15">
+      <c r="B28" s="16">
         <v>4</v>
       </c>
-      <c r="C28" s="15" t="s">
+      <c r="C28" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="D28" s="38">
+      <c r="D28" s="39">
         <f t="shared" si="0"/>
         <v>46095</v>
       </c>
-      <c r="E28" s="16" t="s">
+      <c r="E28" s="17" t="s">
         <v>69</v>
       </c>
-      <c r="F28" s="49" t="s">
+      <c r="F28" s="50" t="s">
         <v>70</v>
       </c>
-      <c r="G28" s="15">
-        <v>2</v>
-      </c>
-      <c r="H28" s="15"/>
-      <c r="I28" s="50" t="s">
+      <c r="G28" s="16">
+        <v>2</v>
+      </c>
+      <c r="H28" s="16"/>
+      <c r="I28" s="51" t="s">
         <v>71</v>
       </c>
-      <c r="J28" s="15" t="s">
+      <c r="J28" s="16" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="29" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A29" s="11">
+      <c r="A29" s="12">
         <v>25</v>
       </c>
-      <c r="B29" s="11">
+      <c r="B29" s="12">
         <v>4</v>
       </c>
-      <c r="C29" s="11" t="s">
+      <c r="C29" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="D29" s="38">
+      <c r="D29" s="39">
         <f t="shared" si="0"/>
         <v>46096</v>
       </c>
-      <c r="E29" s="12" t="s">
+      <c r="E29" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="F29" s="45" t="s">
+      <c r="F29" s="46" t="s">
         <v>72</v>
       </c>
-      <c r="G29" s="11">
-        <v>2</v>
-      </c>
-      <c r="H29" s="11"/>
-      <c r="I29" s="46" t="s">
+      <c r="G29" s="12">
+        <v>2</v>
+      </c>
+      <c r="H29" s="12"/>
+      <c r="I29" s="47" t="s">
         <v>73</v>
       </c>
-      <c r="J29" s="11" t="s">
+      <c r="J29" s="12" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="30" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A30" s="17">
+      <c r="A30" s="18">
         <v>26</v>
       </c>
-      <c r="B30" s="17">
+      <c r="B30" s="18">
         <v>4</v>
       </c>
-      <c r="C30" s="17" t="s">
+      <c r="C30" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="D30" s="38">
+      <c r="D30" s="39">
         <f t="shared" si="0"/>
         <v>46097</v>
       </c>
-      <c r="E30" s="18" t="s">
+      <c r="E30" s="19" t="s">
         <v>74</v>
       </c>
-      <c r="F30" s="51" t="s">
+      <c r="F30" s="52" t="s">
         <v>75</v>
       </c>
-      <c r="G30" s="17">
-        <v>2</v>
-      </c>
-      <c r="H30" s="17"/>
-      <c r="I30" s="52" t="s">
+      <c r="G30" s="18">
+        <v>2</v>
+      </c>
+      <c r="H30" s="18"/>
+      <c r="I30" s="53" t="s">
         <v>76</v>
       </c>
-      <c r="J30" s="17" t="s">
+      <c r="J30" s="18" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="31" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A31" s="9">
+      <c r="A31" s="10">
         <v>27</v>
       </c>
-      <c r="B31" s="9">
+      <c r="B31" s="10">
         <v>4</v>
       </c>
-      <c r="C31" s="9" t="s">
+      <c r="C31" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="D31" s="38">
+      <c r="D31" s="39">
         <f t="shared" si="0"/>
         <v>46098</v>
       </c>
-      <c r="E31" s="10" t="s">
+      <c r="E31" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="F31" s="43" t="s">
+      <c r="F31" s="44" t="s">
         <v>77</v>
       </c>
-      <c r="G31" s="9">
+      <c r="G31" s="10">
         <v>5</v>
       </c>
-      <c r="H31" s="9"/>
-      <c r="I31" s="44" t="s">
+      <c r="H31" s="10"/>
+      <c r="I31" s="45" t="s">
         <v>78</v>
       </c>
-      <c r="J31" s="9" t="s">
+      <c r="J31" s="10" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="32" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A32" s="9">
+      <c r="A32" s="10">
         <v>28</v>
       </c>
-      <c r="B32" s="9">
+      <c r="B32" s="10">
         <v>4</v>
       </c>
-      <c r="C32" s="9" t="s">
+      <c r="C32" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="D32" s="38">
+      <c r="D32" s="39">
         <f t="shared" si="0"/>
         <v>46099</v>
       </c>
-      <c r="E32" s="10" t="s">
+      <c r="E32" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="F32" s="43" t="s">
+      <c r="F32" s="44" t="s">
         <v>79</v>
       </c>
-      <c r="G32" s="9">
+      <c r="G32" s="10">
         <v>5</v>
       </c>
-      <c r="H32" s="9"/>
-      <c r="I32" s="44" t="s">
+      <c r="H32" s="10"/>
+      <c r="I32" s="45" t="s">
         <v>80</v>
       </c>
-      <c r="J32" s="9" t="s">
+      <c r="J32" s="10" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="33" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A33" s="15">
+      <c r="A33" s="16">
         <v>29</v>
       </c>
-      <c r="B33" s="15">
+      <c r="B33" s="16">
         <v>5</v>
       </c>
-      <c r="C33" s="15" t="s">
+      <c r="C33" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="D33" s="38">
+      <c r="D33" s="39">
         <f t="shared" si="0"/>
         <v>46100</v>
       </c>
-      <c r="E33" s="16" t="s">
+      <c r="E33" s="17" t="s">
         <v>69</v>
       </c>
-      <c r="F33" s="49" t="s">
+      <c r="F33" s="50" t="s">
         <v>81</v>
       </c>
-      <c r="G33" s="15">
-        <v>2</v>
-      </c>
-      <c r="H33" s="15"/>
-      <c r="I33" s="50" t="s">
+      <c r="G33" s="16">
+        <v>2</v>
+      </c>
+      <c r="H33" s="16"/>
+      <c r="I33" s="51" t="s">
         <v>82</v>
       </c>
-      <c r="J33" s="15" t="s">
+      <c r="J33" s="16" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="34" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A34" s="17">
+      <c r="A34" s="18">
         <v>30</v>
       </c>
-      <c r="B34" s="17">
+      <c r="B34" s="18">
         <v>5</v>
       </c>
-      <c r="C34" s="17" t="s">
+      <c r="C34" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="D34" s="38">
+      <c r="D34" s="39">
         <f t="shared" si="0"/>
         <v>46101</v>
       </c>
-      <c r="E34" s="18" t="s">
+      <c r="E34" s="19" t="s">
         <v>74</v>
       </c>
-      <c r="F34" s="51" t="s">
+      <c r="F34" s="52" t="s">
         <v>83</v>
       </c>
-      <c r="G34" s="17">
-        <v>2</v>
-      </c>
-      <c r="H34" s="17"/>
-      <c r="I34" s="52" t="s">
+      <c r="G34" s="18">
+        <v>2</v>
+      </c>
+      <c r="H34" s="18"/>
+      <c r="I34" s="53" t="s">
         <v>84</v>
       </c>
-      <c r="J34" s="17" t="s">
+      <c r="J34" s="18" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="35" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A35" s="11">
+      <c r="A35" s="12">
         <v>31</v>
       </c>
-      <c r="B35" s="11">
+      <c r="B35" s="12">
         <v>5</v>
       </c>
-      <c r="C35" s="11" t="s">
+      <c r="C35" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="D35" s="38">
+      <c r="D35" s="39">
         <f t="shared" si="0"/>
         <v>46102</v>
       </c>
-      <c r="E35" s="12" t="s">
+      <c r="E35" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="F35" s="45" t="s">
+      <c r="F35" s="46" t="s">
         <v>85</v>
       </c>
-      <c r="G35" s="11">
-        <v>2</v>
-      </c>
-      <c r="H35" s="11"/>
-      <c r="I35" s="46" t="s">
+      <c r="G35" s="12">
+        <v>2</v>
+      </c>
+      <c r="H35" s="12"/>
+      <c r="I35" s="47" t="s">
         <v>86</v>
       </c>
-      <c r="J35" s="11" t="s">
+      <c r="J35" s="12" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="36" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A36" s="11">
+      <c r="A36" s="12">
         <v>32</v>
       </c>
-      <c r="B36" s="11">
+      <c r="B36" s="12">
         <v>5</v>
       </c>
-      <c r="C36" s="11" t="s">
+      <c r="C36" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="D36" s="38">
+      <c r="D36" s="39">
         <f t="shared" si="0"/>
         <v>46103</v>
       </c>
-      <c r="E36" s="12" t="s">
+      <c r="E36" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="F36" s="45" t="s">
+      <c r="F36" s="46" t="s">
         <v>87</v>
       </c>
-      <c r="G36" s="11">
-        <v>2</v>
-      </c>
-      <c r="H36" s="11"/>
-      <c r="I36" s="46" t="s">
+      <c r="G36" s="12">
+        <v>2</v>
+      </c>
+      <c r="H36" s="12"/>
+      <c r="I36" s="47" t="s">
         <v>88</v>
       </c>
-      <c r="J36" s="11" t="s">
+      <c r="J36" s="12" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="37" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A37" s="11">
+      <c r="A37" s="12">
         <v>33</v>
       </c>
-      <c r="B37" s="11">
+      <c r="B37" s="12">
         <v>5</v>
       </c>
-      <c r="C37" s="11" t="s">
+      <c r="C37" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="D37" s="38">
+      <c r="D37" s="39">
         <f t="shared" si="0"/>
         <v>46104</v>
       </c>
-      <c r="E37" s="12" t="s">
+      <c r="E37" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="F37" s="45" t="s">
+      <c r="F37" s="46" t="s">
         <v>89</v>
       </c>
-      <c r="G37" s="11">
-        <v>2</v>
-      </c>
-      <c r="H37" s="11"/>
-      <c r="I37" s="46" t="s">
+      <c r="G37" s="12">
+        <v>2</v>
+      </c>
+      <c r="H37" s="12"/>
+      <c r="I37" s="47" t="s">
         <v>90</v>
       </c>
-      <c r="J37" s="11" t="s">
+      <c r="J37" s="12" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="38" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A38" s="9">
+      <c r="A38" s="10">
         <v>34</v>
       </c>
-      <c r="B38" s="9">
+      <c r="B38" s="10">
         <v>5</v>
       </c>
-      <c r="C38" s="9" t="s">
+      <c r="C38" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="D38" s="38">
+      <c r="D38" s="39">
         <f t="shared" si="0"/>
         <v>46105</v>
       </c>
-      <c r="E38" s="10" t="s">
+      <c r="E38" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="F38" s="43" t="s">
+      <c r="F38" s="44" t="s">
         <v>91</v>
       </c>
-      <c r="G38" s="9">
+      <c r="G38" s="10">
         <v>5</v>
       </c>
-      <c r="H38" s="9"/>
-      <c r="I38" s="44" t="s">
+      <c r="H38" s="10"/>
+      <c r="I38" s="45" t="s">
         <v>92</v>
       </c>
-      <c r="J38" s="9" t="s">
+      <c r="J38" s="10" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="39" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A39" s="9">
+      <c r="A39" s="10">
         <v>35</v>
       </c>
-      <c r="B39" s="9">
+      <c r="B39" s="10">
         <v>5</v>
       </c>
-      <c r="C39" s="9" t="s">
+      <c r="C39" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="D39" s="38">
+      <c r="D39" s="39">
         <f t="shared" si="0"/>
         <v>46106</v>
       </c>
-      <c r="E39" s="10" t="s">
+      <c r="E39" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="F39" s="43" t="s">
+      <c r="F39" s="44" t="s">
         <v>93</v>
       </c>
-      <c r="G39" s="9">
+      <c r="G39" s="10">
         <v>5</v>
       </c>
-      <c r="H39" s="9"/>
-      <c r="I39" s="44" t="s">
+      <c r="H39" s="10"/>
+      <c r="I39" s="45" t="s">
         <v>94</v>
       </c>
-      <c r="J39" s="9" t="s">
+      <c r="J39" s="10" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="40" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A40" s="15">
+      <c r="A40" s="16">
         <v>36</v>
       </c>
-      <c r="B40" s="15">
+      <c r="B40" s="16">
         <v>6</v>
       </c>
-      <c r="C40" s="15" t="s">
+      <c r="C40" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="D40" s="38">
+      <c r="D40" s="39">
         <f t="shared" si="0"/>
         <v>46107</v>
       </c>
-      <c r="E40" s="16" t="s">
+      <c r="E40" s="17" t="s">
         <v>69</v>
       </c>
-      <c r="F40" s="49" t="s">
+      <c r="F40" s="50" t="s">
         <v>95</v>
       </c>
-      <c r="G40" s="15">
-        <v>2</v>
-      </c>
-      <c r="H40" s="15"/>
-      <c r="I40" s="50" t="s">
+      <c r="G40" s="16">
+        <v>2</v>
+      </c>
+      <c r="H40" s="16"/>
+      <c r="I40" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="J40" s="15" t="s">
+      <c r="J40" s="16" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="41" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A41" s="15">
+      <c r="A41" s="16">
         <v>37</v>
       </c>
-      <c r="B41" s="15">
+      <c r="B41" s="16">
         <v>6</v>
       </c>
-      <c r="C41" s="15" t="s">
+      <c r="C41" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="D41" s="38">
+      <c r="D41" s="39">
         <f t="shared" si="0"/>
         <v>46108</v>
       </c>
-      <c r="E41" s="16" t="s">
+      <c r="E41" s="17" t="s">
         <v>69</v>
       </c>
-      <c r="F41" s="49" t="s">
+      <c r="F41" s="50" t="s">
         <v>97</v>
       </c>
-      <c r="G41" s="15">
-        <v>2</v>
-      </c>
-      <c r="H41" s="15"/>
-      <c r="I41" s="50" t="s">
+      <c r="G41" s="16">
+        <v>2</v>
+      </c>
+      <c r="H41" s="16"/>
+      <c r="I41" s="51" t="s">
         <v>98</v>
       </c>
-      <c r="J41" s="15" t="s">
+      <c r="J41" s="16" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="42" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A42" s="15">
+      <c r="A42" s="16">
         <v>38</v>
       </c>
-      <c r="B42" s="15">
+      <c r="B42" s="16">
         <v>6</v>
       </c>
-      <c r="C42" s="15" t="s">
+      <c r="C42" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="D42" s="38">
+      <c r="D42" s="39">
         <f t="shared" si="0"/>
         <v>46109</v>
       </c>
-      <c r="E42" s="16" t="s">
+      <c r="E42" s="17" t="s">
         <v>69</v>
       </c>
-      <c r="F42" s="49" t="s">
+      <c r="F42" s="50" t="s">
         <v>99</v>
       </c>
-      <c r="G42" s="15">
-        <v>2</v>
-      </c>
-      <c r="H42" s="15"/>
-      <c r="I42" s="50" t="s">
+      <c r="G42" s="16">
+        <v>2</v>
+      </c>
+      <c r="H42" s="16"/>
+      <c r="I42" s="51" t="s">
         <v>100</v>
       </c>
-      <c r="J42" s="15" t="s">
+      <c r="J42" s="16" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="43" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A43" s="17">
+      <c r="A43" s="18">
         <v>39</v>
       </c>
-      <c r="B43" s="17">
+      <c r="B43" s="18">
         <v>6</v>
       </c>
-      <c r="C43" s="17" t="s">
+      <c r="C43" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="D43" s="38">
+      <c r="D43" s="39">
         <f t="shared" si="0"/>
         <v>46110</v>
       </c>
-      <c r="E43" s="18" t="s">
+      <c r="E43" s="19" t="s">
         <v>74</v>
       </c>
-      <c r="F43" s="51" t="s">
+      <c r="F43" s="52" t="s">
         <v>101</v>
       </c>
-      <c r="G43" s="17">
-        <v>2</v>
-      </c>
-      <c r="H43" s="17"/>
-      <c r="I43" s="52" t="s">
+      <c r="G43" s="18">
+        <v>2</v>
+      </c>
+      <c r="H43" s="18"/>
+      <c r="I43" s="53" t="s">
         <v>102</v>
       </c>
-      <c r="J43" s="17" t="s">
+      <c r="J43" s="18" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="44" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A44" s="17">
+      <c r="A44" s="18">
         <v>40</v>
       </c>
-      <c r="B44" s="17">
+      <c r="B44" s="18">
         <v>6</v>
       </c>
-      <c r="C44" s="17" t="s">
+      <c r="C44" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="D44" s="38">
+      <c r="D44" s="39">
         <f t="shared" si="0"/>
         <v>46111</v>
       </c>
-      <c r="E44" s="18" t="s">
+      <c r="E44" s="19" t="s">
         <v>74</v>
       </c>
-      <c r="F44" s="51" t="s">
+      <c r="F44" s="52" t="s">
         <v>103</v>
       </c>
-      <c r="G44" s="17">
-        <v>2</v>
-      </c>
-      <c r="H44" s="17"/>
-      <c r="I44" s="52" t="s">
+      <c r="G44" s="18">
+        <v>2</v>
+      </c>
+      <c r="H44" s="18"/>
+      <c r="I44" s="53" t="s">
         <v>104</v>
       </c>
-      <c r="J44" s="17" t="s">
+      <c r="J44" s="18" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="45" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A45" s="9">
+      <c r="A45" s="10">
         <v>41</v>
       </c>
-      <c r="B45" s="9">
+      <c r="B45" s="10">
         <v>6</v>
       </c>
-      <c r="C45" s="9" t="s">
+      <c r="C45" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="D45" s="38">
+      <c r="D45" s="39">
         <f t="shared" si="0"/>
         <v>46112</v>
       </c>
-      <c r="E45" s="10" t="s">
+      <c r="E45" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="F45" s="43" t="s">
+      <c r="F45" s="44" t="s">
         <v>105</v>
       </c>
-      <c r="G45" s="9">
+      <c r="G45" s="10">
         <v>5</v>
       </c>
-      <c r="H45" s="9"/>
-      <c r="I45" s="44" t="s">
+      <c r="H45" s="10"/>
+      <c r="I45" s="45" t="s">
         <v>106</v>
       </c>
-      <c r="J45" s="9" t="s">
+      <c r="J45" s="10" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="46" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A46" s="9">
+      <c r="A46" s="10">
         <v>42</v>
       </c>
-      <c r="B46" s="9">
+      <c r="B46" s="10">
         <v>6</v>
       </c>
-      <c r="C46" s="9" t="s">
+      <c r="C46" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="D46" s="38">
+      <c r="D46" s="39">
         <f t="shared" si="0"/>
         <v>46113</v>
       </c>
-      <c r="E46" s="10" t="s">
+      <c r="E46" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="F46" s="43" t="s">
+      <c r="F46" s="44" t="s">
         <v>107</v>
       </c>
-      <c r="G46" s="9">
+      <c r="G46" s="10">
         <v>5</v>
       </c>
-      <c r="H46" s="9"/>
-      <c r="I46" s="44" t="s">
+      <c r="H46" s="10"/>
+      <c r="I46" s="45" t="s">
         <v>108</v>
       </c>
-      <c r="J46" s="9" t="s">
+      <c r="J46" s="10" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="47" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A47" s="17">
+      <c r="A47" s="18">
         <v>43</v>
       </c>
-      <c r="B47" s="17">
+      <c r="B47" s="18">
         <v>7</v>
       </c>
-      <c r="C47" s="17" t="s">
+      <c r="C47" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="D47" s="38">
+      <c r="D47" s="39">
         <f t="shared" si="0"/>
         <v>46114</v>
       </c>
-      <c r="E47" s="18" t="s">
+      <c r="E47" s="19" t="s">
         <v>74</v>
       </c>
-      <c r="F47" s="51" t="s">
+      <c r="F47" s="52" t="s">
         <v>109</v>
       </c>
-      <c r="G47" s="17">
-        <v>2</v>
-      </c>
-      <c r="H47" s="17"/>
-      <c r="I47" s="52" t="s">
+      <c r="G47" s="18">
+        <v>2</v>
+      </c>
+      <c r="H47" s="18"/>
+      <c r="I47" s="53" t="s">
         <v>110</v>
       </c>
-      <c r="J47" s="17" t="s">
+      <c r="J47" s="18" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="48" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A48" s="17">
+      <c r="A48" s="18">
         <v>44</v>
       </c>
-      <c r="B48" s="17">
+      <c r="B48" s="18">
         <v>7</v>
       </c>
-      <c r="C48" s="17" t="s">
+      <c r="C48" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="D48" s="38">
+      <c r="D48" s="39">
         <f t="shared" si="0"/>
         <v>46115</v>
       </c>
-      <c r="E48" s="18" t="s">
+      <c r="E48" s="19" t="s">
         <v>74</v>
       </c>
-      <c r="F48" s="51" t="s">
+      <c r="F48" s="52" t="s">
         <v>111</v>
       </c>
-      <c r="G48" s="17">
-        <v>2</v>
-      </c>
-      <c r="H48" s="17"/>
-      <c r="I48" s="52" t="s">
+      <c r="G48" s="18">
+        <v>2</v>
+      </c>
+      <c r="H48" s="18"/>
+      <c r="I48" s="53" t="s">
         <v>112</v>
       </c>
-      <c r="J48" s="17" t="s">
+      <c r="J48" s="18" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="49" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A49" s="17">
+      <c r="A49" s="18">
         <v>45</v>
       </c>
-      <c r="B49" s="17">
+      <c r="B49" s="18">
         <v>7</v>
       </c>
-      <c r="C49" s="17" t="s">
+      <c r="C49" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="D49" s="38">
+      <c r="D49" s="39">
         <f t="shared" si="0"/>
         <v>46116</v>
       </c>
-      <c r="E49" s="18" t="s">
+      <c r="E49" s="19" t="s">
         <v>74</v>
       </c>
-      <c r="F49" s="51" t="s">
+      <c r="F49" s="52" t="s">
         <v>113</v>
       </c>
-      <c r="G49" s="17">
-        <v>2</v>
-      </c>
-      <c r="H49" s="17"/>
-      <c r="I49" s="52" t="s">
+      <c r="G49" s="18">
+        <v>2</v>
+      </c>
+      <c r="H49" s="18"/>
+      <c r="I49" s="53" t="s">
         <v>114</v>
       </c>
-      <c r="J49" s="17" t="s">
+      <c r="J49" s="18" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="50" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A50" s="17">
+      <c r="A50" s="18">
         <v>46</v>
       </c>
-      <c r="B50" s="17">
+      <c r="B50" s="18">
         <v>7</v>
       </c>
-      <c r="C50" s="17" t="s">
+      <c r="C50" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="D50" s="38">
+      <c r="D50" s="39">
         <f t="shared" si="0"/>
         <v>46117</v>
       </c>
-      <c r="E50" s="18" t="s">
+      <c r="E50" s="19" t="s">
         <v>74</v>
       </c>
-      <c r="F50" s="51" t="s">
+      <c r="F50" s="52" t="s">
         <v>115</v>
       </c>
-      <c r="G50" s="17">
-        <v>2</v>
-      </c>
-      <c r="H50" s="17"/>
-      <c r="I50" s="52" t="s">
+      <c r="G50" s="18">
+        <v>2</v>
+      </c>
+      <c r="H50" s="18"/>
+      <c r="I50" s="53" t="s">
         <v>116</v>
       </c>
-      <c r="J50" s="17" t="s">
+      <c r="J50" s="18" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="51" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A51" s="17">
+      <c r="A51" s="18">
         <v>47</v>
       </c>
-      <c r="B51" s="17">
+      <c r="B51" s="18">
         <v>7</v>
       </c>
-      <c r="C51" s="17" t="s">
+      <c r="C51" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="D51" s="38">
+      <c r="D51" s="39">
         <f t="shared" si="0"/>
         <v>46118</v>
       </c>
-      <c r="E51" s="18" t="s">
+      <c r="E51" s="19" t="s">
         <v>74</v>
       </c>
-      <c r="F51" s="51" t="s">
+      <c r="F51" s="52" t="s">
         <v>117</v>
       </c>
-      <c r="G51" s="17">
-        <v>2</v>
-      </c>
-      <c r="H51" s="17"/>
-      <c r="I51" s="52" t="s">
+      <c r="G51" s="18">
+        <v>2</v>
+      </c>
+      <c r="H51" s="18"/>
+      <c r="I51" s="53" t="s">
         <v>118</v>
       </c>
-      <c r="J51" s="17" t="s">
+      <c r="J51" s="18" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="52" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A52" s="9">
+      <c r="A52" s="10">
         <v>48</v>
       </c>
-      <c r="B52" s="9">
+      <c r="B52" s="10">
         <v>7</v>
       </c>
-      <c r="C52" s="9" t="s">
+      <c r="C52" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="D52" s="38">
+      <c r="D52" s="39">
         <f t="shared" si="0"/>
         <v>46119</v>
       </c>
-      <c r="E52" s="10" t="s">
+      <c r="E52" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="F52" s="43" t="s">
+      <c r="F52" s="44" t="s">
         <v>119</v>
       </c>
-      <c r="G52" s="9">
+      <c r="G52" s="10">
         <v>5</v>
       </c>
-      <c r="H52" s="9"/>
-      <c r="I52" s="44" t="s">
+      <c r="H52" s="10"/>
+      <c r="I52" s="45" t="s">
         <v>120</v>
       </c>
-      <c r="J52" s="9" t="s">
+      <c r="J52" s="10" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="53" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A53" s="9">
+      <c r="A53" s="10">
         <v>49</v>
       </c>
-      <c r="B53" s="9">
+      <c r="B53" s="10">
         <v>7</v>
       </c>
-      <c r="C53" s="9" t="s">
+      <c r="C53" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="D53" s="38">
+      <c r="D53" s="39">
         <f t="shared" si="0"/>
         <v>46120</v>
       </c>
-      <c r="E53" s="10" t="s">
+      <c r="E53" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="F53" s="43" t="s">
+      <c r="F53" s="44" t="s">
         <v>121</v>
       </c>
-      <c r="G53" s="9">
+      <c r="G53" s="10">
         <v>5</v>
       </c>
-      <c r="H53" s="9"/>
-      <c r="I53" s="44" t="s">
+      <c r="H53" s="10"/>
+      <c r="I53" s="45" t="s">
         <v>122</v>
       </c>
-      <c r="J53" s="9" t="s">
+      <c r="J53" s="10" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="54" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A54" s="17">
+      <c r="A54" s="18">
         <v>50</v>
       </c>
-      <c r="B54" s="17">
+      <c r="B54" s="18">
         <v>8</v>
       </c>
-      <c r="C54" s="17" t="s">
+      <c r="C54" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="D54" s="38">
+      <c r="D54" s="39">
         <f t="shared" si="0"/>
         <v>46121</v>
       </c>
-      <c r="E54" s="18" t="s">
+      <c r="E54" s="19" t="s">
         <v>74</v>
       </c>
-      <c r="F54" s="51" t="s">
+      <c r="F54" s="52" t="s">
         <v>123</v>
       </c>
-      <c r="G54" s="17">
-        <v>2</v>
-      </c>
-      <c r="H54" s="17"/>
-      <c r="I54" s="52" t="s">
+      <c r="G54" s="18">
+        <v>2</v>
+      </c>
+      <c r="H54" s="18"/>
+      <c r="I54" s="53" t="s">
         <v>124</v>
       </c>
-      <c r="J54" s="17" t="s">
+      <c r="J54" s="18" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="55" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A55" s="17">
+      <c r="A55" s="18">
         <v>51</v>
       </c>
-      <c r="B55" s="17">
+      <c r="B55" s="18">
         <v>8</v>
       </c>
-      <c r="C55" s="17" t="s">
+      <c r="C55" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="D55" s="38">
+      <c r="D55" s="39">
         <f t="shared" si="0"/>
         <v>46122</v>
       </c>
-      <c r="E55" s="18" t="s">
+      <c r="E55" s="19" t="s">
         <v>74</v>
       </c>
-      <c r="F55" s="51" t="s">
+      <c r="F55" s="52" t="s">
         <v>125</v>
       </c>
-      <c r="G55" s="17">
-        <v>2</v>
-      </c>
-      <c r="H55" s="17"/>
-      <c r="I55" s="52" t="s">
+      <c r="G55" s="18">
+        <v>2</v>
+      </c>
+      <c r="H55" s="18"/>
+      <c r="I55" s="53" t="s">
         <v>126</v>
       </c>
-      <c r="J55" s="17" t="s">
+      <c r="J55" s="18" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="56" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A56" s="17">
+      <c r="A56" s="18">
         <v>52</v>
       </c>
-      <c r="B56" s="17">
+      <c r="B56" s="18">
         <v>8</v>
       </c>
-      <c r="C56" s="17" t="s">
+      <c r="C56" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="D56" s="38">
+      <c r="D56" s="39">
         <f t="shared" si="0"/>
         <v>46123</v>
       </c>
-      <c r="E56" s="18" t="s">
+      <c r="E56" s="19" t="s">
         <v>74</v>
       </c>
-      <c r="F56" s="51" t="s">
+      <c r="F56" s="52" t="s">
         <v>127</v>
       </c>
-      <c r="G56" s="17">
-        <v>2</v>
-      </c>
-      <c r="H56" s="17"/>
-      <c r="I56" s="52" t="s">
+      <c r="G56" s="18">
+        <v>2</v>
+      </c>
+      <c r="H56" s="18"/>
+      <c r="I56" s="53" t="s">
         <v>128</v>
       </c>
-      <c r="J56" s="17" t="s">
+      <c r="J56" s="18" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="57" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A57" s="17">
+      <c r="A57" s="18">
         <v>53</v>
       </c>
-      <c r="B57" s="17">
+      <c r="B57" s="18">
         <v>8</v>
       </c>
-      <c r="C57" s="17" t="s">
+      <c r="C57" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="D57" s="38">
+      <c r="D57" s="39">
         <f t="shared" si="0"/>
         <v>46124</v>
       </c>
-      <c r="E57" s="18" t="s">
+      <c r="E57" s="19" t="s">
         <v>74</v>
       </c>
-      <c r="F57" s="51" t="s">
+      <c r="F57" s="52" t="s">
         <v>129</v>
       </c>
-      <c r="G57" s="17">
-        <v>2</v>
-      </c>
-      <c r="H57" s="17"/>
-      <c r="I57" s="52" t="s">
+      <c r="G57" s="18">
+        <v>2</v>
+      </c>
+      <c r="H57" s="18"/>
+      <c r="I57" s="53" t="s">
         <v>130</v>
       </c>
-      <c r="J57" s="17" t="s">
+      <c r="J57" s="18" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="58" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A58" s="17">
+      <c r="A58" s="18">
         <v>54</v>
       </c>
-      <c r="B58" s="17">
+      <c r="B58" s="18">
         <v>8</v>
       </c>
-      <c r="C58" s="17" t="s">
+      <c r="C58" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="D58" s="38">
+      <c r="D58" s="39">
         <f t="shared" si="0"/>
         <v>46125</v>
       </c>
-      <c r="E58" s="18" t="s">
+      <c r="E58" s="19" t="s">
         <v>74</v>
       </c>
-      <c r="F58" s="51" t="s">
+      <c r="F58" s="52" t="s">
         <v>131</v>
       </c>
-      <c r="G58" s="17">
-        <v>2</v>
-      </c>
-      <c r="H58" s="17"/>
-      <c r="I58" s="52" t="s">
+      <c r="G58" s="18">
+        <v>2</v>
+      </c>
+      <c r="H58" s="18"/>
+      <c r="I58" s="53" t="s">
         <v>132</v>
       </c>
-      <c r="J58" s="17" t="s">
+      <c r="J58" s="18" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="59" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A59" s="9">
+      <c r="A59" s="10">
         <v>55</v>
       </c>
-      <c r="B59" s="9">
+      <c r="B59" s="10">
         <v>8</v>
       </c>
-      <c r="C59" s="9" t="s">
+      <c r="C59" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="D59" s="38">
+      <c r="D59" s="39">
         <f t="shared" si="0"/>
         <v>46126</v>
       </c>
-      <c r="E59" s="10" t="s">
+      <c r="E59" s="11" t="s">
         <v>133</v>
       </c>
-      <c r="F59" s="43" t="s">
+      <c r="F59" s="44" t="s">
         <v>134</v>
       </c>
-      <c r="G59" s="9">
+      <c r="G59" s="10">
         <v>5</v>
       </c>
-      <c r="H59" s="9"/>
-      <c r="I59" s="44" t="s">
+      <c r="H59" s="10"/>
+      <c r="I59" s="45" t="s">
         <v>135</v>
       </c>
-      <c r="J59" s="9" t="s">
+      <c r="J59" s="10" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="60" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A60" s="9">
+      <c r="A60" s="10">
         <v>56</v>
       </c>
-      <c r="B60" s="9">
+      <c r="B60" s="10">
         <v>8</v>
       </c>
-      <c r="C60" s="9" t="s">
+      <c r="C60" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="D60" s="38">
+      <c r="D60" s="39">
         <f t="shared" si="0"/>
         <v>46127</v>
       </c>
-      <c r="E60" s="10" t="s">
+      <c r="E60" s="11" t="s">
         <v>133</v>
       </c>
-      <c r="F60" s="43" t="s">
+      <c r="F60" s="44" t="s">
         <v>136</v>
       </c>
-      <c r="G60" s="9">
+      <c r="G60" s="10">
         <v>5</v>
       </c>
-      <c r="H60" s="9"/>
-      <c r="I60" s="44" t="s">
+      <c r="H60" s="10"/>
+      <c r="I60" s="45" t="s">
         <v>137</v>
       </c>
-      <c r="J60" s="9" t="s">
+      <c r="J60" s="10" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="61" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A61" s="19">
+      <c r="A61" s="20">
         <v>57</v>
       </c>
-      <c r="B61" s="19">
+      <c r="B61" s="20">
         <v>9</v>
       </c>
-      <c r="C61" s="19" t="s">
+      <c r="C61" s="20" t="s">
         <v>11</v>
       </c>
-      <c r="D61" s="38">
+      <c r="D61" s="39">
         <f t="shared" si="0"/>
         <v>46128</v>
       </c>
-      <c r="E61" s="20" t="s">
+      <c r="E61" s="21" t="s">
         <v>133</v>
       </c>
-      <c r="F61" s="53" t="s">
+      <c r="F61" s="54" t="s">
         <v>138</v>
       </c>
-      <c r="G61" s="19">
-        <v>2</v>
-      </c>
-      <c r="H61" s="19"/>
-      <c r="I61" s="54" t="s">
+      <c r="G61" s="20">
+        <v>2</v>
+      </c>
+      <c r="H61" s="20"/>
+      <c r="I61" s="55" t="s">
         <v>139</v>
       </c>
-      <c r="J61" s="19" t="s">
+      <c r="J61" s="20" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="62" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A62" s="19">
+      <c r="A62" s="20">
         <v>58</v>
       </c>
-      <c r="B62" s="19">
+      <c r="B62" s="20">
         <v>9</v>
       </c>
-      <c r="C62" s="19" t="s">
+      <c r="C62" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="D62" s="38">
+      <c r="D62" s="39">
         <f t="shared" si="0"/>
         <v>46129</v>
       </c>
-      <c r="E62" s="20" t="s">
+      <c r="E62" s="21" t="s">
         <v>133</v>
       </c>
-      <c r="F62" s="53" t="s">
+      <c r="F62" s="54" t="s">
         <v>140</v>
       </c>
-      <c r="G62" s="19">
-        <v>2</v>
-      </c>
-      <c r="H62" s="19"/>
-      <c r="I62" s="54" t="s">
+      <c r="G62" s="20">
+        <v>2</v>
+      </c>
+      <c r="H62" s="20"/>
+      <c r="I62" s="55" t="s">
         <v>141</v>
       </c>
-      <c r="J62" s="19" t="s">
+      <c r="J62" s="20" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="63" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A63" s="17">
+      <c r="A63" s="18">
         <v>59</v>
       </c>
-      <c r="B63" s="17">
+      <c r="B63" s="18">
         <v>9</v>
       </c>
-      <c r="C63" s="17" t="s">
+      <c r="C63" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="D63" s="38">
+      <c r="D63" s="39">
         <f t="shared" si="0"/>
         <v>46130</v>
       </c>
-      <c r="E63" s="18" t="s">
+      <c r="E63" s="19" t="s">
         <v>74</v>
       </c>
-      <c r="F63" s="51" t="s">
+      <c r="F63" s="52" t="s">
         <v>142</v>
       </c>
-      <c r="G63" s="17">
-        <v>2</v>
-      </c>
-      <c r="H63" s="17"/>
-      <c r="I63" s="52" t="s">
+      <c r="G63" s="18">
+        <v>2</v>
+      </c>
+      <c r="H63" s="18"/>
+      <c r="I63" s="53" t="s">
         <v>143</v>
       </c>
-      <c r="J63" s="17" t="s">
+      <c r="J63" s="18" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="64" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A64" s="17">
+      <c r="A64" s="18">
         <v>60</v>
       </c>
-      <c r="B64" s="17">
+      <c r="B64" s="18">
         <v>9</v>
       </c>
-      <c r="C64" s="17" t="s">
+      <c r="C64" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="D64" s="38">
+      <c r="D64" s="39">
         <f t="shared" si="0"/>
         <v>46131</v>
       </c>
-      <c r="E64" s="18" t="s">
+      <c r="E64" s="19" t="s">
         <v>74</v>
       </c>
-      <c r="F64" s="51" t="s">
+      <c r="F64" s="52" t="s">
         <v>144</v>
       </c>
-      <c r="G64" s="17">
-        <v>2</v>
-      </c>
-      <c r="H64" s="17"/>
-      <c r="I64" s="52" t="s">
+      <c r="G64" s="18">
+        <v>2</v>
+      </c>
+      <c r="H64" s="18"/>
+      <c r="I64" s="53" t="s">
         <v>145</v>
       </c>
-      <c r="J64" s="17" t="s">
+      <c r="J64" s="18" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="65" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A65" s="17">
+      <c r="A65" s="18">
         <v>61</v>
       </c>
-      <c r="B65" s="17">
+      <c r="B65" s="18">
         <v>9</v>
       </c>
-      <c r="C65" s="17" t="s">
+      <c r="C65" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="D65" s="38">
+      <c r="D65" s="39">
         <f t="shared" si="0"/>
         <v>46132</v>
       </c>
-      <c r="E65" s="18" t="s">
+      <c r="E65" s="19" t="s">
         <v>74</v>
       </c>
-      <c r="F65" s="51" t="s">
+      <c r="F65" s="52" t="s">
         <v>146</v>
       </c>
-      <c r="G65" s="17">
-        <v>2</v>
-      </c>
-      <c r="H65" s="17"/>
-      <c r="I65" s="52" t="s">
+      <c r="G65" s="18">
+        <v>2</v>
+      </c>
+      <c r="H65" s="18"/>
+      <c r="I65" s="53" t="s">
         <v>147</v>
       </c>
-      <c r="J65" s="17" t="s">
+      <c r="J65" s="18" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="66" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A66" s="9">
+      <c r="A66" s="10">
         <v>62</v>
       </c>
-      <c r="B66" s="9">
+      <c r="B66" s="10">
         <v>9</v>
       </c>
-      <c r="C66" s="9" t="s">
+      <c r="C66" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="D66" s="38">
+      <c r="D66" s="39">
         <f t="shared" si="0"/>
         <v>46133</v>
       </c>
-      <c r="E66" s="10" t="s">
+      <c r="E66" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="F66" s="43" t="s">
+      <c r="F66" s="44" t="s">
         <v>148</v>
       </c>
-      <c r="G66" s="9">
+      <c r="G66" s="10">
         <v>5</v>
       </c>
-      <c r="H66" s="9"/>
-      <c r="I66" s="44" t="s">
+      <c r="H66" s="10"/>
+      <c r="I66" s="45" t="s">
         <v>149</v>
       </c>
-      <c r="J66" s="9" t="s">
+      <c r="J66" s="10" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="67" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A67" s="9">
+      <c r="A67" s="10">
         <v>63</v>
       </c>
-      <c r="B67" s="9">
+      <c r="B67" s="10">
         <v>9</v>
       </c>
-      <c r="C67" s="9" t="s">
+      <c r="C67" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="D67" s="38">
+      <c r="D67" s="39">
         <f t="shared" si="0"/>
         <v>46134</v>
       </c>
-      <c r="E67" s="10" t="s">
+      <c r="E67" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="F67" s="43" t="s">
+      <c r="F67" s="44" t="s">
         <v>150</v>
       </c>
-      <c r="G67" s="9">
+      <c r="G67" s="10">
         <v>5</v>
       </c>
-      <c r="H67" s="9"/>
-      <c r="I67" s="44" t="s">
+      <c r="H67" s="10"/>
+      <c r="I67" s="45" t="s">
         <v>151</v>
       </c>
-      <c r="J67" s="9" t="s">
+      <c r="J67" s="10" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="68" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A68" s="17">
+      <c r="A68" s="18">
         <v>64</v>
       </c>
-      <c r="B68" s="17">
+      <c r="B68" s="18">
         <v>10</v>
       </c>
-      <c r="C68" s="17" t="s">
+      <c r="C68" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="D68" s="38">
+      <c r="D68" s="39">
         <f t="shared" si="0"/>
         <v>46135</v>
       </c>
-      <c r="E68" s="18" t="s">
+      <c r="E68" s="19" t="s">
         <v>74</v>
       </c>
-      <c r="F68" s="51" t="s">
+      <c r="F68" s="52" t="s">
         <v>152</v>
       </c>
-      <c r="G68" s="17">
-        <v>2</v>
-      </c>
-      <c r="H68" s="17"/>
-      <c r="I68" s="52" t="s">
+      <c r="G68" s="18">
+        <v>2</v>
+      </c>
+      <c r="H68" s="18"/>
+      <c r="I68" s="53" t="s">
         <v>153</v>
       </c>
-      <c r="J68" s="17" t="s">
+      <c r="J68" s="18" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="69" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A69" s="17">
+      <c r="A69" s="18">
         <v>65</v>
       </c>
-      <c r="B69" s="17">
+      <c r="B69" s="18">
         <v>10</v>
       </c>
-      <c r="C69" s="17" t="s">
+      <c r="C69" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="D69" s="38">
+      <c r="D69" s="39">
         <f t="shared" si="0"/>
         <v>46136</v>
       </c>
-      <c r="E69" s="18" t="s">
+      <c r="E69" s="19" t="s">
         <v>74</v>
       </c>
-      <c r="F69" s="51" t="s">
+      <c r="F69" s="52" t="s">
         <v>154</v>
       </c>
-      <c r="G69" s="17">
-        <v>2</v>
-      </c>
-      <c r="H69" s="17"/>
-      <c r="I69" s="52" t="s">
+      <c r="G69" s="18">
+        <v>2</v>
+      </c>
+      <c r="H69" s="18"/>
+      <c r="I69" s="53" t="s">
         <v>155</v>
       </c>
-      <c r="J69" s="17" t="s">
+      <c r="J69" s="18" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="71" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="F71" s="21" t="s">
+      <c r="F71" s="22" t="s">
         <v>156</v>
       </c>
-      <c r="G71" s="21">
+      <c r="G71" s="22">
         <f>SUM(G5:G69)</f>
         <v>184</v>
       </c>
@@ -3935,253 +3938,253 @@
       <c r="F1" s="1"/>
     </row>
     <row r="3" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="22" t="s">
+      <c r="B3" s="23" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="22" t="s">
+      <c r="C3" s="23" t="s">
         <v>158</v>
       </c>
-      <c r="D3" s="22" t="s">
+      <c r="D3" s="23" t="s">
         <v>159</v>
       </c>
-      <c r="E3" s="22" t="s">
+      <c r="E3" s="23" t="s">
         <v>160</v>
       </c>
-      <c r="F3" s="22" t="s">
+      <c r="F3" s="23" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="23">
+      <c r="A4" s="24">
         <v>1</v>
       </c>
-      <c r="B4" s="24" t="s">
+      <c r="B4" s="25" t="s">
         <v>162</v>
       </c>
-      <c r="C4" s="25" t="s">
+      <c r="C4" s="26" t="s">
         <v>33</v>
       </c>
-      <c r="D4" s="26">
+      <c r="D4" s="27">
         <v>20</v>
       </c>
-      <c r="E4" s="27">
-        <v>2</v>
-      </c>
-      <c r="F4" s="28" t="s">
+      <c r="E4" s="28">
+        <v>2</v>
+      </c>
+      <c r="F4" s="29" t="s">
         <v>163</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="23">
-        <v>2</v>
-      </c>
-      <c r="B5" s="29" t="s">
+      <c r="A5" s="24">
+        <v>2</v>
+      </c>
+      <c r="B5" s="30" t="s">
         <v>164</v>
       </c>
-      <c r="C5" s="25" t="s">
+      <c r="C5" s="26" t="s">
         <v>48</v>
       </c>
-      <c r="D5" s="26">
+      <c r="D5" s="27">
         <v>20</v>
       </c>
-      <c r="E5" s="30">
+      <c r="E5" s="31">
         <v>5</v>
       </c>
-      <c r="F5" s="28" t="s">
+      <c r="F5" s="29" t="s">
         <v>165</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="23">
+      <c r="A6" s="24">
         <v>3</v>
       </c>
-      <c r="B6" s="29" t="s">
+      <c r="B6" s="30" t="s">
         <v>166</v>
       </c>
-      <c r="C6" s="25" t="s">
+      <c r="C6" s="26" t="s">
         <v>63</v>
       </c>
-      <c r="D6" s="26">
+      <c r="D6" s="27">
         <v>20</v>
       </c>
-      <c r="E6" s="27">
-        <v>2</v>
-      </c>
-      <c r="F6" s="28" t="s">
+      <c r="E6" s="28">
+        <v>2</v>
+      </c>
+      <c r="F6" s="29" t="s">
         <v>167</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="23">
+      <c r="A7" s="24">
         <v>4</v>
       </c>
-      <c r="B7" s="29" t="s">
+      <c r="B7" s="30" t="s">
         <v>168</v>
       </c>
-      <c r="C7" s="25" t="s">
+      <c r="C7" s="26" t="s">
         <v>79</v>
       </c>
-      <c r="D7" s="26">
+      <c r="D7" s="27">
         <v>20</v>
       </c>
-      <c r="E7" s="27">
+      <c r="E7" s="28">
         <v>0</v>
       </c>
-      <c r="F7" s="28" t="s">
+      <c r="F7" s="29" t="s">
         <v>169</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="23">
+      <c r="A8" s="24">
         <v>5</v>
       </c>
-      <c r="B8" s="31" t="s">
+      <c r="B8" s="32" t="s">
         <v>170</v>
       </c>
-      <c r="C8" s="25" t="s">
+      <c r="C8" s="26" t="s">
         <v>93</v>
       </c>
-      <c r="D8" s="26">
+      <c r="D8" s="27">
         <v>20</v>
       </c>
-      <c r="E8" s="27">
+      <c r="E8" s="28">
         <v>0</v>
       </c>
-      <c r="F8" s="28" t="s">
+      <c r="F8" s="29" t="s">
         <v>171</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="23">
+      <c r="A9" s="24">
         <v>6</v>
       </c>
-      <c r="B9" s="32" t="s">
+      <c r="B9" s="33" t="s">
         <v>172</v>
       </c>
-      <c r="C9" s="25" t="s">
+      <c r="C9" s="26" t="s">
         <v>107</v>
       </c>
-      <c r="D9" s="26">
+      <c r="D9" s="27">
         <v>20</v>
       </c>
-      <c r="E9" s="30">
+      <c r="E9" s="31">
         <v>0</v>
       </c>
-      <c r="F9" s="28" t="s">
+      <c r="F9" s="29" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="23">
+      <c r="A10" s="24">
         <v>7</v>
       </c>
-      <c r="B10" s="33" t="s">
+      <c r="B10" s="34" t="s">
         <v>74</v>
       </c>
-      <c r="C10" s="25" t="s">
+      <c r="C10" s="26" t="s">
         <v>121</v>
       </c>
-      <c r="D10" s="26">
+      <c r="D10" s="27">
         <v>20</v>
       </c>
-      <c r="E10" s="30">
+      <c r="E10" s="31">
         <v>0</v>
       </c>
-      <c r="F10" s="28" t="s">
+      <c r="F10" s="29" t="s">
         <v>174</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="23">
+      <c r="A11" s="24">
         <v>8</v>
       </c>
-      <c r="B11" s="34" t="s">
+      <c r="B11" s="35" t="s">
         <v>175</v>
       </c>
-      <c r="C11" s="25" t="s">
+      <c r="C11" s="26" t="s">
         <v>136</v>
       </c>
-      <c r="D11" s="26">
+      <c r="D11" s="27">
         <v>20</v>
       </c>
-      <c r="E11" s="27">
+      <c r="E11" s="28">
         <v>0</v>
       </c>
-      <c r="F11" s="28" t="s">
+      <c r="F11" s="29" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="23">
+      <c r="A12" s="24">
         <v>9</v>
       </c>
-      <c r="B12" s="32" t="s">
+      <c r="B12" s="33" t="s">
         <v>175</v>
       </c>
-      <c r="C12" s="25" t="s">
+      <c r="C12" s="26" t="s">
         <v>150</v>
       </c>
-      <c r="D12" s="26">
+      <c r="D12" s="27">
         <v>20</v>
       </c>
-      <c r="E12" s="30">
+      <c r="E12" s="31">
         <v>0</v>
       </c>
-      <c r="F12" s="28" t="s">
+      <c r="F12" s="29" t="s">
         <v>177</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="23">
+      <c r="A13" s="24">
         <v>10</v>
       </c>
-      <c r="B13" s="32" t="s">
+      <c r="B13" s="33" t="s">
         <v>74</v>
       </c>
-      <c r="C13" s="25" t="s">
+      <c r="C13" s="26" t="s">
         <v>154</v>
       </c>
-      <c r="D13" s="26">
+      <c r="D13" s="27">
         <v>4</v>
       </c>
-      <c r="E13" s="30">
+      <c r="E13" s="31">
         <v>0</v>
       </c>
-      <c r="F13" s="28" t="s">
+      <c r="F13" s="29" t="s">
         <v>178</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="23"/>
-      <c r="B14" s="32"/>
-      <c r="C14" s="25"/>
-      <c r="D14" s="26"/>
-      <c r="E14" s="30"/>
-      <c r="F14" s="28"/>
+      <c r="A14" s="24"/>
+      <c r="B14" s="33"/>
+      <c r="C14" s="26"/>
+      <c r="D14" s="27"/>
+      <c r="E14" s="31"/>
+      <c r="F14" s="29"/>
     </row>
     <row r="15" spans="1:6" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="23"/>
-      <c r="B15" s="35"/>
-      <c r="C15" s="25"/>
-      <c r="D15" s="26"/>
-      <c r="E15" s="30"/>
-      <c r="F15" s="28"/>
+      <c r="A15" s="24"/>
+      <c r="B15" s="36"/>
+      <c r="C15" s="26"/>
+      <c r="D15" s="27"/>
+      <c r="E15" s="31"/>
+      <c r="F15" s="29"/>
     </row>
     <row r="16" spans="1:6" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="23"/>
-      <c r="B16" s="31"/>
-      <c r="C16" s="25"/>
-      <c r="D16" s="26"/>
-      <c r="E16" s="30"/>
-      <c r="F16" s="28"/>
+      <c r="A16" s="24"/>
+      <c r="B16" s="32"/>
+      <c r="C16" s="26"/>
+      <c r="D16" s="27"/>
+      <c r="E16" s="31"/>
+      <c r="F16" s="29"/>
     </row>
     <row r="17" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C17" s="36"/>
-      <c r="D17" s="23"/>
-      <c r="E17" s="37"/>
+      <c r="C17" s="37"/>
+      <c r="D17" s="24"/>
+      <c r="E17" s="38"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>